<commit_message>
TO RERUN SCRIPTS; changed minor error in ground truth and MERCEC calculation error, along with xlsx caching
</commit_message>
<xml_diff>
--- a/Scoring Logic and Documentation/method/merec_weights_summary.xlsx
+++ b/Scoring Logic and Documentation/method/merec_weights_summary.xlsx
@@ -473,16 +473,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.228272</v>
+        <v>0.164213</v>
       </c>
       <c r="E2" t="n">
-        <v>0.080147</v>
+        <v>0.158337</v>
       </c>
       <c r="F2" t="n">
         <v>0.3</v>
       </c>
       <c r="G2" t="n">
-        <v>-0.071728</v>
+        <v>-0.135787</v>
       </c>
       <c r="H2" t="n">
         <v>44</v>
@@ -503,16 +503,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.205089</v>
+        <v>0.107178</v>
       </c>
       <c r="E3" t="n">
-        <v>0.070517</v>
+        <v>0.114416</v>
       </c>
       <c r="F3" t="n">
         <v>0.35</v>
       </c>
       <c r="G3" t="n">
-        <v>-0.144911</v>
+        <v>-0.242822</v>
       </c>
       <c r="H3" t="n">
         <v>48</v>
@@ -533,16 +533,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.28362</v>
+        <v>0.437285</v>
       </c>
       <c r="E4" t="n">
-        <v>0.175317</v>
+        <v>0.255249</v>
       </c>
       <c r="F4" t="n">
         <v>0.2</v>
       </c>
       <c r="G4" t="n">
-        <v>0.08362</v>
+        <v>0.237285</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
@@ -563,16 +563,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.28302</v>
+        <v>0.291324</v>
       </c>
       <c r="E5" t="n">
-        <v>0.123339</v>
+        <v>0.240534</v>
       </c>
       <c r="F5" t="n">
         <v>0.15</v>
       </c>
       <c r="G5" t="n">
-        <v>0.13302</v>
+        <v>0.141324</v>
       </c>
       <c r="H5" t="n">
         <v>52</v>
@@ -593,16 +593,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.184696</v>
+        <v>0.155571</v>
       </c>
       <c r="E6" t="n">
-        <v>0.062568</v>
+        <v>0.144712</v>
       </c>
       <c r="F6" t="n">
         <v>0.3</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.115304</v>
+        <v>-0.144429</v>
       </c>
       <c r="H6" t="n">
         <v>17</v>
@@ -623,16 +623,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.16058</v>
+        <v>0.127537</v>
       </c>
       <c r="E7" t="n">
-        <v>0.030637</v>
+        <v>0.09975100000000001</v>
       </c>
       <c r="F7" t="n">
         <v>0.35</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.18942</v>
+        <v>-0.222463</v>
       </c>
       <c r="H7" t="n">
         <v>17</v>
@@ -653,16 +653,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.46978</v>
+        <v>0.673507</v>
       </c>
       <c r="E8" t="n">
-        <v>0.08612300000000001</v>
+        <v>0.222379</v>
       </c>
       <c r="F8" t="n">
         <v>0.2</v>
       </c>
       <c r="G8" t="n">
-        <v>0.26978</v>
+        <v>0.473507</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -683,16 +683,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.184944</v>
+        <v>0.043385</v>
       </c>
       <c r="E9" t="n">
-        <v>0.066071</v>
+        <v>0.057996</v>
       </c>
       <c r="F9" t="n">
         <v>0.15</v>
       </c>
       <c r="G9" t="n">
-        <v>0.034944</v>
+        <v>-0.106615</v>
       </c>
       <c r="H9" t="n">
         <v>52</v>
@@ -713,16 +713,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.25081</v>
+        <v>0.126796</v>
       </c>
       <c r="E10" t="n">
-        <v>0.075609</v>
+        <v>0.174136</v>
       </c>
       <c r="F10" t="n">
         <v>0.3</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.04919</v>
+        <v>-0.173204</v>
       </c>
       <c r="H10" t="n">
         <v>27</v>
@@ -743,16 +743,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.259931</v>
+        <v>0.056389</v>
       </c>
       <c r="E11" t="n">
-        <v>0.08022700000000001</v>
+        <v>0.137667</v>
       </c>
       <c r="F11" t="n">
         <v>0.35</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.090069</v>
+        <v>-0.293611</v>
       </c>
       <c r="H11" t="n">
         <v>31</v>
@@ -773,16 +773,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.163514</v>
+        <v>0.32746</v>
       </c>
       <c r="E12" t="n">
-        <v>0.104637</v>
+        <v>0.13695</v>
       </c>
       <c r="F12" t="n">
         <v>0.2</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.036486</v>
+        <v>0.12746</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -803,16 +803,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.325745</v>
+        <v>0.489354</v>
       </c>
       <c r="E13" t="n">
-        <v>0.119374</v>
+        <v>0.1771</v>
       </c>
       <c r="F13" t="n">
         <v>0.15</v>
       </c>
       <c r="G13" t="n">
-        <v>0.175745</v>
+        <v>0.339354</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -833,16 +833,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.258463</v>
+        <v>0.222423</v>
       </c>
       <c r="E14" t="n">
-        <v>0.081882</v>
+        <v>0.139298</v>
       </c>
       <c r="F14" t="n">
         <v>0.3</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.041537</v>
+        <v>-0.07757699999999999</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -863,16 +863,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.196251</v>
+        <v>0.143267</v>
       </c>
       <c r="E15" t="n">
-        <v>0.046097</v>
+        <v>0.072005</v>
       </c>
       <c r="F15" t="n">
         <v>0.35</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.153749</v>
+        <v>-0.206733</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -893,16 +893,16 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.184343</v>
+        <v>0.258223</v>
       </c>
       <c r="E16" t="n">
-        <v>0.111358</v>
+        <v>0.150291</v>
       </c>
       <c r="F16" t="n">
         <v>0.2</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.015657</v>
+        <v>0.058223</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -923,16 +923,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.360943</v>
+        <v>0.376087</v>
       </c>
       <c r="E17" t="n">
-        <v>0.0994</v>
+        <v>0.159695</v>
       </c>
       <c r="F17" t="n">
         <v>0.15</v>
       </c>
       <c r="G17" t="n">
-        <v>0.210943</v>
+        <v>0.226087</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>

</xml_diff>